<commit_message>
fix SV, VV LVALH, PNL
</commit_message>
<xml_diff>
--- a/БД/funcs/SV_LVALH.xlsx
+++ b/БД/funcs/SV_LVALH.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="233">
   <si>
     <t>Modbus RTU</t>
   </si>
@@ -558,12 +558,6 @@
     <t>CALH1_OvrlExtSign_Ctrl</t>
   </si>
   <si>
-    <t xml:space="preserve">Контроль положения переключателя аварийной деблокировки </t>
-  </si>
-  <si>
-    <t>CALH1_SwPosEmergUnblk_Ctrl</t>
-  </si>
-  <si>
     <t>Parameter</t>
   </si>
   <si>
@@ -657,9 +651,6 @@
     <t>Контр_общ_вн_сигн</t>
   </si>
   <si>
-    <t>Контр_пол_ав_дебл</t>
-  </si>
-  <si>
     <t>SV_LVALH</t>
   </si>
   <si>
@@ -693,13 +684,7 @@
     <t>Сраб УРОВ на себя</t>
   </si>
   <si>
-    <t>Положение переключателя аварийной деблокировки 1</t>
-  </si>
-  <si>
     <t>SwPosOfEmergUnblk1</t>
-  </si>
-  <si>
-    <t>Положение переключателя аварийной деблокировки 2</t>
   </si>
   <si>
     <t>Полож.пер.ав.дебл.2</t>
@@ -713,12 +698,39 @@
   <si>
     <t>input</t>
   </si>
+  <si>
+    <t>Контроль положения переключателя 1 аварийной деблокировки</t>
+  </si>
+  <si>
+    <t>Контр_пол_ав_дебл_1</t>
+  </si>
+  <si>
+    <t>CALH1_SwPosEmergUnblk1_Ctrl</t>
+  </si>
+  <si>
+    <t>Контроль положения переключателя 2 аварийной деблокировки</t>
+  </si>
+  <si>
+    <t>Контр_пол_ав_дебл_2</t>
+  </si>
+  <si>
+    <t>SGF8</t>
+  </si>
+  <si>
+    <t>CALH1_SwPosEmergUnblk2_Ctrl</t>
+  </si>
+  <si>
+    <t>Положение переключателя 1 аварийной деблокировки</t>
+  </si>
+  <si>
+    <t>Положение переключателя 2 аварийной деблокировки</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -791,15 +803,8 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial Narrow"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -839,6 +844,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -904,7 +915,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1092,41 +1103,74 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1653,13 +1697,13 @@
         <v>47</v>
       </c>
       <c r="AV2" s="49" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="AW2" s="49" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="AX2" s="49" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="AY2" s="14"/>
       <c r="AZ2" s="13" t="s">
@@ -18010,7 +18054,7 @@
     <row r="3" spans="1:16379" s="66" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="52"/>
       <c r="B3" s="52" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C3" s="53"/>
       <c r="D3" s="54"/>
@@ -18227,7 +18271,7 @@
         <v>0</v>
       </c>
       <c r="AV4" s="25">
-        <f t="shared" ref="AV3:AV40" si="3">BIN2DEC(CONCATENATE(0,0,0,0,AR4,AS4,AT4,AU4))</f>
+        <f t="shared" ref="AV4:AV40" si="3">BIN2DEC(CONCATENATE(0,0,0,0,AR4,AS4,AT4,AU4))</f>
         <v>0</v>
       </c>
       <c r="AW4" s="25">
@@ -18502,13 +18546,13 @@
       <c r="C7" s="19"/>
       <c r="D7" s="33"/>
       <c r="E7" s="21" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H7" s="21"/>
       <c r="I7" s="21">
@@ -18520,7 +18564,7 @@
         <v>Ср.сигн. ДЗ-фф 4ст.</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="L7" s="22" t="s">
         <v>62</v>
@@ -18868,13 +18912,13 @@
       <c r="C10" s="19"/>
       <c r="D10" s="33"/>
       <c r="E10" s="21" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H10" s="21"/>
       <c r="I10" s="21">
@@ -18886,7 +18930,7 @@
         <v>Ср.сигн. ТЗНП 3 ст.</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="L10" s="22" t="s">
         <v>62</v>
@@ -18990,13 +19034,13 @@
       <c r="C11" s="19"/>
       <c r="D11" s="33"/>
       <c r="E11" s="21" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H11" s="21"/>
       <c r="I11" s="21">
@@ -19008,7 +19052,7 @@
         <v>Ср.сигн. ТЗНП 4 ст.</v>
       </c>
       <c r="K11" s="18" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="L11" s="22" t="s">
         <v>62</v>
@@ -19112,13 +19156,13 @@
       <c r="C12" s="19"/>
       <c r="D12" s="33"/>
       <c r="E12" s="21" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H12" s="21"/>
       <c r="I12" s="21">
@@ -19600,13 +19644,13 @@
       <c r="C16" s="19"/>
       <c r="D16" s="33"/>
       <c r="E16" s="21" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H16" s="21"/>
       <c r="I16" s="21">
@@ -19618,7 +19662,7 @@
         <v>Ср.сигн. МТЗ 4 ст.</v>
       </c>
       <c r="K16" s="18" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="L16" s="22" t="s">
         <v>62</v>
@@ -20088,13 +20132,13 @@
       <c r="C20" s="19"/>
       <c r="D20" s="33"/>
       <c r="E20" s="21" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F20" s="21" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="G20" s="21" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H20" s="21"/>
       <c r="I20" s="21">
@@ -20106,7 +20150,7 @@
         <v>Неиспр. ЛЗШ</v>
       </c>
       <c r="K20" s="18" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="L20" s="22" t="s">
         <v>62</v>
@@ -20210,13 +20254,13 @@
       <c r="C21" s="19"/>
       <c r="D21" s="33"/>
       <c r="E21" s="21" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H21" s="21"/>
       <c r="I21" s="21">
@@ -20332,13 +20376,13 @@
       <c r="C22" s="19"/>
       <c r="D22" s="33"/>
       <c r="E22" s="21" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="G22" s="21" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H22" s="21"/>
       <c r="I22" s="21">
@@ -20820,13 +20864,13 @@
       <c r="C26" s="19"/>
       <c r="D26" s="33"/>
       <c r="E26" s="21" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F26" s="21" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H26" s="21"/>
       <c r="I26" s="21">
@@ -21064,13 +21108,13 @@
       <c r="C28" s="19"/>
       <c r="D28" s="33"/>
       <c r="E28" s="51" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F28" s="51" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="G28" s="51" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="H28" s="21"/>
       <c r="I28" s="21">
@@ -22276,249 +22320,249 @@
       </c>
       <c r="BH37" s="30"/>
     </row>
-    <row r="38" spans="1:60" s="81" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="69"/>
-      <c r="B38" s="69" t="s">
-        <v>228</v>
-      </c>
-      <c r="C38" s="70"/>
-      <c r="D38" s="71"/>
-      <c r="E38" s="72" t="s">
-        <v>222</v>
-      </c>
-      <c r="F38" s="72" t="s">
-        <v>226</v>
-      </c>
-      <c r="G38" s="72" t="s">
-        <v>226</v>
-      </c>
-      <c r="H38" s="72"/>
-      <c r="I38" s="72">
+    <row r="38" spans="1:60" s="92" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="78"/>
+      <c r="B38" s="78" t="s">
+        <v>223</v>
+      </c>
+      <c r="C38" s="79"/>
+      <c r="D38" s="80"/>
+      <c r="E38" s="81" t="s">
+        <v>231</v>
+      </c>
+      <c r="F38" s="81" t="s">
+        <v>221</v>
+      </c>
+      <c r="G38" s="81" t="s">
+        <v>221</v>
+      </c>
+      <c r="H38" s="81"/>
+      <c r="I38" s="81">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="J38" s="72" t="str">
+      <c r="J38" s="81" t="str">
         <f t="shared" si="1"/>
         <v>Полож.пер.ав.дебл.1</v>
       </c>
-      <c r="K38" s="69" t="s">
-        <v>223</v>
-      </c>
-      <c r="L38" s="73" t="s">
+      <c r="K38" s="78" t="s">
+        <v>219</v>
+      </c>
+      <c r="L38" s="82" t="s">
         <v>62</v>
       </c>
-      <c r="M38" s="70" t="s">
+      <c r="M38" s="79" t="s">
         <v>63</v>
       </c>
-      <c r="N38" s="70" t="s">
+      <c r="N38" s="79" t="s">
         <v>64</v>
       </c>
-      <c r="O38" s="70"/>
-      <c r="P38" s="74"/>
-      <c r="Q38" s="74"/>
-      <c r="R38" s="70" t="s">
+      <c r="O38" s="79"/>
+      <c r="P38" s="83"/>
+      <c r="Q38" s="83"/>
+      <c r="R38" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="S38" s="70" t="s">
+      <c r="S38" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="T38" s="70" t="s">
+      <c r="T38" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="U38" s="70" t="s">
+      <c r="U38" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="V38" s="70"/>
-      <c r="W38" s="70"/>
-      <c r="X38" s="70" t="s">
+      <c r="V38" s="79"/>
+      <c r="W38" s="79"/>
+      <c r="X38" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="Y38" s="70">
+      <c r="Y38" s="79">
         <v>0</v>
       </c>
-      <c r="Z38" s="75"/>
-      <c r="AA38" s="76">
+      <c r="Z38" s="84"/>
+      <c r="AA38" s="85">
         <v>0</v>
       </c>
-      <c r="AB38" s="76"/>
-      <c r="AC38" s="76"/>
-      <c r="AD38" s="76"/>
-      <c r="AE38" s="76"/>
-      <c r="AF38" s="76">
+      <c r="AB38" s="85"/>
+      <c r="AC38" s="85"/>
+      <c r="AD38" s="85"/>
+      <c r="AE38" s="85"/>
+      <c r="AF38" s="85">
         <v>0</v>
       </c>
-      <c r="AG38" s="76">
+      <c r="AG38" s="85">
         <v>0</v>
       </c>
-      <c r="AH38" s="76">
+      <c r="AH38" s="85">
         <v>0</v>
       </c>
-      <c r="AI38" s="77"/>
-      <c r="AJ38" s="78"/>
-      <c r="AK38" s="78"/>
-      <c r="AL38" s="78"/>
-      <c r="AM38" s="78"/>
-      <c r="AN38" s="78"/>
-      <c r="AO38" s="78"/>
-      <c r="AP38" s="78"/>
-      <c r="AQ38" s="78"/>
-      <c r="AR38" s="76">
+      <c r="AI38" s="86"/>
+      <c r="AJ38" s="87"/>
+      <c r="AK38" s="87"/>
+      <c r="AL38" s="87"/>
+      <c r="AM38" s="87"/>
+      <c r="AN38" s="87"/>
+      <c r="AO38" s="87"/>
+      <c r="AP38" s="87"/>
+      <c r="AQ38" s="87"/>
+      <c r="AR38" s="85">
         <v>0</v>
       </c>
-      <c r="AS38" s="76">
+      <c r="AS38" s="85">
         <v>0</v>
       </c>
-      <c r="AT38" s="76">
+      <c r="AT38" s="85">
         <v>0</v>
       </c>
-      <c r="AU38" s="76">
+      <c r="AU38" s="85">
         <v>0</v>
       </c>
-      <c r="AV38" s="76">
+      <c r="AV38" s="85">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AW38" s="76">
+      <c r="AW38" s="85">
         <v>0</v>
       </c>
-      <c r="AX38" s="76">
+      <c r="AX38" s="85">
         <v>0</v>
       </c>
-      <c r="AY38" s="76"/>
-      <c r="AZ38" s="74"/>
-      <c r="BA38" s="76"/>
-      <c r="BB38" s="76"/>
-      <c r="BC38" s="76"/>
-      <c r="BD38" s="76"/>
-      <c r="BE38" s="76"/>
-      <c r="BF38" s="76"/>
-      <c r="BG38" s="79" t="str">
+      <c r="AY38" s="85"/>
+      <c r="AZ38" s="83"/>
+      <c r="BA38" s="85"/>
+      <c r="BB38" s="85"/>
+      <c r="BC38" s="88"/>
+      <c r="BD38" s="85"/>
+      <c r="BE38" s="89"/>
+      <c r="BF38" s="85"/>
+      <c r="BG38" s="90" t="str">
         <f t="shared" si="2"/>
-        <v>description: "Полож.пер.ав.дебл.1", note: "Положение переключателя аварийной деблокировки 1", group: "input", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 0</v>
-      </c>
-      <c r="BH38" s="80"/>
+        <v>description: "Полож.пер.ав.дебл.1", note: "Положение переключателя 1 аварийной деблокировки", group: "input", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 0</v>
+      </c>
+      <c r="BH38" s="91"/>
     </row>
-    <row r="39" spans="1:60" s="81" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="69"/>
-      <c r="B39" s="69" t="s">
-        <v>228</v>
-      </c>
-      <c r="C39" s="70"/>
-      <c r="D39" s="71"/>
-      <c r="E39" s="72" t="s">
-        <v>224</v>
-      </c>
-      <c r="F39" s="72" t="s">
-        <v>225</v>
-      </c>
-      <c r="G39" s="72" t="s">
-        <v>225</v>
-      </c>
-      <c r="H39" s="72"/>
-      <c r="I39" s="72">
-        <f t="shared" ref="I39" si="20">LEN(F39)</f>
+    <row r="39" spans="1:60" s="92" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="78"/>
+      <c r="B39" s="78" t="s">
+        <v>223</v>
+      </c>
+      <c r="C39" s="79"/>
+      <c r="D39" s="80"/>
+      <c r="E39" s="81" t="s">
+        <v>232</v>
+      </c>
+      <c r="F39" s="81" t="s">
+        <v>220</v>
+      </c>
+      <c r="G39" s="81" t="s">
+        <v>220</v>
+      </c>
+      <c r="H39" s="81"/>
+      <c r="I39" s="81">
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="J39" s="72" t="str">
-        <f t="shared" ref="J39" si="21">IF(LEN(F39)&lt;=$J$1,F39,"")</f>
+      <c r="J39" s="81" t="str">
+        <f t="shared" si="1"/>
         <v>Полож.пер.ав.дебл.2</v>
       </c>
-      <c r="K39" s="69" t="s">
-        <v>227</v>
-      </c>
-      <c r="L39" s="73" t="s">
+      <c r="K39" s="78" t="s">
+        <v>222</v>
+      </c>
+      <c r="L39" s="82" t="s">
         <v>62</v>
       </c>
-      <c r="M39" s="70" t="s">
+      <c r="M39" s="79" t="s">
         <v>63</v>
       </c>
-      <c r="N39" s="70" t="s">
+      <c r="N39" s="79" t="s">
         <v>64</v>
       </c>
-      <c r="O39" s="70"/>
-      <c r="P39" s="74"/>
-      <c r="Q39" s="74"/>
-      <c r="R39" s="70" t="s">
+      <c r="O39" s="79"/>
+      <c r="P39" s="83"/>
+      <c r="Q39" s="83"/>
+      <c r="R39" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="S39" s="70" t="s">
+      <c r="S39" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="T39" s="70" t="s">
+      <c r="T39" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="U39" s="70" t="s">
+      <c r="U39" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="V39" s="70"/>
-      <c r="W39" s="70"/>
-      <c r="X39" s="70" t="s">
+      <c r="V39" s="79"/>
+      <c r="W39" s="79"/>
+      <c r="X39" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="Y39" s="70">
+      <c r="Y39" s="79">
         <v>0</v>
       </c>
-      <c r="Z39" s="75"/>
-      <c r="AA39" s="76">
+      <c r="Z39" s="84"/>
+      <c r="AA39" s="85">
         <v>0</v>
       </c>
-      <c r="AB39" s="76"/>
-      <c r="AC39" s="76"/>
-      <c r="AD39" s="76"/>
-      <c r="AE39" s="76"/>
-      <c r="AF39" s="76">
+      <c r="AB39" s="85"/>
+      <c r="AC39" s="85"/>
+      <c r="AD39" s="85"/>
+      <c r="AE39" s="85"/>
+      <c r="AF39" s="85">
         <v>0</v>
       </c>
-      <c r="AG39" s="76">
+      <c r="AG39" s="85">
         <v>0</v>
       </c>
-      <c r="AH39" s="76">
+      <c r="AH39" s="85">
         <v>0</v>
       </c>
-      <c r="AI39" s="77"/>
-      <c r="AJ39" s="78"/>
-      <c r="AK39" s="78"/>
-      <c r="AL39" s="78"/>
-      <c r="AM39" s="78"/>
-      <c r="AN39" s="78"/>
-      <c r="AO39" s="78"/>
-      <c r="AP39" s="78"/>
-      <c r="AQ39" s="78"/>
-      <c r="AR39" s="76">
+      <c r="AI39" s="86"/>
+      <c r="AJ39" s="87"/>
+      <c r="AK39" s="87"/>
+      <c r="AL39" s="87"/>
+      <c r="AM39" s="87"/>
+      <c r="AN39" s="87"/>
+      <c r="AO39" s="87"/>
+      <c r="AP39" s="87"/>
+      <c r="AQ39" s="87"/>
+      <c r="AR39" s="85">
         <v>0</v>
       </c>
-      <c r="AS39" s="76">
+      <c r="AS39" s="85">
         <v>0</v>
       </c>
-      <c r="AT39" s="76">
+      <c r="AT39" s="85">
         <v>0</v>
       </c>
-      <c r="AU39" s="76">
+      <c r="AU39" s="85">
         <v>0</v>
       </c>
-      <c r="AV39" s="76">
-        <f t="shared" ref="AV39" si="22">BIN2DEC(CONCATENATE(0,0,0,0,AR39,AS39,AT39,AU39))</f>
+      <c r="AV39" s="85">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AW39" s="76">
+      <c r="AW39" s="85">
         <v>0</v>
       </c>
-      <c r="AX39" s="76">
+      <c r="AX39" s="85">
         <v>0</v>
       </c>
-      <c r="AY39" s="76"/>
-      <c r="AZ39" s="74"/>
-      <c r="BA39" s="76"/>
-      <c r="BB39" s="76"/>
-      <c r="BC39" s="76"/>
-      <c r="BD39" s="76"/>
-      <c r="BE39" s="76"/>
-      <c r="BF39" s="76"/>
-      <c r="BG39" s="79" t="str">
-        <f t="shared" ref="BG39" si="23">CONCATENATE("description: """,F39,"""", ", ", "note: """,E39,"""",", ","group: """, B39, """",", ","minValue: ", S39,", ","maxValue: ", T39,", ","step: ", U39,", ","units: """, R39, """",", ","defaultValue: ", X39,", ","eventRegistration: ", Y39,)</f>
-        <v>description: "Полож.пер.ав.дебл.2", note: "Положение переключателя аварийной деблокировки 2", group: "input", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 0</v>
-      </c>
-      <c r="BH39" s="80"/>
+      <c r="AY39" s="85"/>
+      <c r="AZ39" s="83"/>
+      <c r="BA39" s="85"/>
+      <c r="BB39" s="85"/>
+      <c r="BC39" s="88"/>
+      <c r="BD39" s="85"/>
+      <c r="BE39" s="89"/>
+      <c r="BF39" s="85"/>
+      <c r="BG39" s="90" t="str">
+        <f t="shared" si="2"/>
+        <v>description: "Полож.пер.ав.дебл.2", note: "Положение переключателя 2 аварийной деблокировки", group: "input", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 0</v>
+      </c>
+      <c r="BH39" s="91"/>
     </row>
     <row r="40" spans="1:60" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="18"/>
@@ -26631,13 +26675,13 @@
         <v>47</v>
       </c>
       <c r="AV2" s="49" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="AW2" s="49" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="AX2" s="49" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="AY2" s="14"/>
       <c r="AZ2" s="13" t="s">
@@ -42988,7 +43032,7 @@
     <row r="3" spans="1:16379" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18"/>
       <c r="B3" s="48" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="33" t="s">
@@ -43110,7 +43154,7 @@
     <row r="4" spans="1:16379" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="18"/>
       <c r="B4" s="48" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C4" s="25"/>
       <c r="D4" s="33" t="s">
@@ -43240,14 +43284,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:XEY9"/>
+  <dimension ref="A1:XEY10"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="58.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="72.140625" style="2" customWidth="1"/>
     <col min="6" max="6" width="22" style="2" customWidth="1" outlineLevel="1"/>
     <col min="7" max="7" width="19.5703125" style="2" bestFit="1" customWidth="1" outlineLevel="1"/>
     <col min="8" max="8" width="40.28515625" style="2" bestFit="1" customWidth="1" outlineLevel="1"/>
@@ -59864,11 +59908,11 @@
         <v>153</v>
       </c>
       <c r="I3" s="21">
-        <f t="shared" ref="I3:I9" si="0">LEN(F3)</f>
+        <f t="shared" ref="I3:I10" si="0">LEN(F3)</f>
         <v>11</v>
       </c>
       <c r="J3" s="21" t="str">
-        <f t="shared" ref="J3:J9" si="1">IF(LEN(F3)&lt;=$J$1,F3,"")</f>
+        <f t="shared" ref="J3:J10" si="1">IF(LEN(F3)&lt;=$J$1,F3,"")</f>
         <v>Контр_цепей</v>
       </c>
       <c r="K3" s="18" t="s">
@@ -59947,7 +59991,7 @@
         <v>0</v>
       </c>
       <c r="AV3" s="25">
-        <f t="shared" ref="AV3:AV9" si="2">BIN2DEC(CONCATENATE(0,0,0,0,AR3,AS3,AT3,AU3))</f>
+        <f t="shared" ref="AV3:AV10" si="2">BIN2DEC(CONCATENATE(0,0,0,0,AR3,AS3,AT3,AU3))</f>
         <v>0</v>
       </c>
       <c r="AW3" s="25" t="s">
@@ -59963,7 +60007,7 @@
       <c r="BE3" s="25"/>
       <c r="BF3" s="25"/>
       <c r="BG3" s="29" t="str">
-        <f t="shared" ref="BG3:BG9" si="3">CONCATENATE("description: """,F3,"""", ", ", "note: """,E3,"""",", ","group: """, B3, """",", ","minValue: ", S3,", ","maxValue: ", T3,", ","step: ", U3,", ","units: """, R3, """",", ","defaultValue: ", X3,", ","eventRegistration: ", Y3,)</f>
+        <f t="shared" ref="BG3:BG10" si="3">CONCATENATE("description: """,F3,"""", ", ", "note: """,E3,"""",", ","group: """, B3, """",", ","minValue: ", S3,", ","maxValue: ", T3,", ","step: ", U3,", ","units: """, R3, """",", ","defaultValue: ", X3,", ","eventRegistration: ", Y3,)</f>
         <v>description: "Контр_цепей", note: "Контроль выходных цепей", group: "setting", minValue: 0, maxValue: 1, step: 1, units: "null", defaultValue: 0, eventRegistration: 0</v>
       </c>
     </row>
@@ -60355,7 +60399,7 @@
         <v>173</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G7" s="21" t="s">
         <v>158</v>
@@ -60480,7 +60524,7 @@
         <v>175</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="G8" s="21" t="s">
         <v>159</v>
@@ -60592,129 +60636,254 @@
         <v>description: "Контр_общ_вн_сигн", note: "Контроль общего внешнего сигнала", group: "setting", minValue: 0, maxValue: 1, step: 1, units: "null", defaultValue: 0, eventRegistration: 0</v>
       </c>
     </row>
-    <row r="9" spans="1:16379" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18" t="s">
+    <row r="9" spans="1:16379" s="38" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="69"/>
+      <c r="B9" s="69" t="s">
         <v>151</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="33" t="s">
+      <c r="C9" s="70"/>
+      <c r="D9" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="E9" s="21" t="s">
-        <v>177</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>210</v>
-      </c>
-      <c r="G9" s="21" t="s">
+      <c r="E9" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="F9" s="77" t="s">
+        <v>225</v>
+      </c>
+      <c r="G9" s="77" t="s">
         <v>162</v>
       </c>
-      <c r="H9" s="21" t="s">
+      <c r="H9" s="71" t="s">
         <v>153</v>
       </c>
-      <c r="I9" s="21">
+      <c r="I9" s="71">
         <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="J9" s="21" t="str">
+        <v>19</v>
+      </c>
+      <c r="J9" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>Контр_пол_ав_дебл</v>
-      </c>
-      <c r="K9" s="18" t="s">
-        <v>178</v>
-      </c>
-      <c r="L9" s="22" t="s">
+        <v>Контр_пол_ав_дебл_1</v>
+      </c>
+      <c r="K9" s="69" t="s">
+        <v>226</v>
+      </c>
+      <c r="L9" s="72" t="s">
         <v>62</v>
       </c>
-      <c r="M9" s="19" t="s">
+      <c r="M9" s="70" t="s">
         <v>64</v>
       </c>
-      <c r="N9" s="19" t="s">
+      <c r="N9" s="70" t="s">
         <v>64</v>
       </c>
-      <c r="O9" s="19"/>
-      <c r="P9" s="23">
+      <c r="O9" s="70"/>
+      <c r="P9" s="73">
         <v>0</v>
       </c>
-      <c r="Q9" s="23"/>
-      <c r="R9" s="19" t="s">
+      <c r="Q9" s="73"/>
+      <c r="R9" s="70" t="s">
         <v>65</v>
       </c>
-      <c r="S9" s="19">
+      <c r="S9" s="70">
         <v>0</v>
       </c>
-      <c r="T9" s="19">
+      <c r="T9" s="70">
         <v>1</v>
       </c>
-      <c r="U9" s="19">
+      <c r="U9" s="70">
         <v>1</v>
       </c>
-      <c r="V9" s="19"/>
-      <c r="W9" s="19"/>
-      <c r="X9" s="19">
+      <c r="V9" s="70"/>
+      <c r="W9" s="70"/>
+      <c r="X9" s="70">
         <v>0</v>
       </c>
-      <c r="Y9" s="19">
+      <c r="Y9" s="70">
         <v>0</v>
       </c>
-      <c r="Z9" s="24"/>
-      <c r="AA9" s="25">
+      <c r="Z9" s="74"/>
+      <c r="AA9" s="75">
         <v>0</v>
       </c>
-      <c r="AB9" s="25"/>
-      <c r="AC9" s="25"/>
-      <c r="AD9" s="25"/>
-      <c r="AE9" s="25"/>
-      <c r="AF9" s="25">
+      <c r="AB9" s="75"/>
+      <c r="AC9" s="75"/>
+      <c r="AD9" s="75"/>
+      <c r="AE9" s="75"/>
+      <c r="AF9" s="75">
         <v>0</v>
       </c>
-      <c r="AG9" s="25">
+      <c r="AG9" s="75">
         <v>0</v>
       </c>
-      <c r="AH9" s="25">
+      <c r="AH9" s="75">
         <v>0</v>
       </c>
-      <c r="AI9" s="25"/>
-      <c r="AJ9" s="25"/>
-      <c r="AK9" s="25"/>
-      <c r="AL9" s="25"/>
-      <c r="AM9" s="25"/>
-      <c r="AN9" s="25"/>
-      <c r="AO9" s="25"/>
-      <c r="AP9" s="25"/>
-      <c r="AQ9" s="25"/>
-      <c r="AR9" s="25">
+      <c r="AI9" s="75"/>
+      <c r="AJ9" s="75"/>
+      <c r="AK9" s="75"/>
+      <c r="AL9" s="75"/>
+      <c r="AM9" s="75"/>
+      <c r="AN9" s="75"/>
+      <c r="AO9" s="75"/>
+      <c r="AP9" s="75"/>
+      <c r="AQ9" s="75"/>
+      <c r="AR9" s="75">
         <v>0</v>
       </c>
-      <c r="AS9" s="25">
+      <c r="AS9" s="75">
         <v>0</v>
       </c>
-      <c r="AT9" s="25">
+      <c r="AT9" s="75">
         <v>0</v>
       </c>
-      <c r="AU9" s="25">
+      <c r="AU9" s="75">
         <v>0</v>
       </c>
-      <c r="AV9" s="25">
+      <c r="AV9" s="75">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="AW9" s="25" t="s">
+      <c r="AW9" s="75" t="s">
         <v>154</v>
       </c>
-      <c r="AX9" s="25"/>
-      <c r="AY9" s="23"/>
-      <c r="AZ9" s="25"/>
-      <c r="BA9" s="25"/>
-      <c r="BB9" s="25"/>
-      <c r="BC9" s="25"/>
-      <c r="BD9" s="25"/>
-      <c r="BE9" s="25"/>
-      <c r="BF9" s="25"/>
-      <c r="BG9" s="29" t="str">
+      <c r="AX9" s="75"/>
+      <c r="AY9" s="73"/>
+      <c r="AZ9" s="75"/>
+      <c r="BA9" s="75"/>
+      <c r="BB9" s="75"/>
+      <c r="BC9" s="75"/>
+      <c r="BD9" s="75"/>
+      <c r="BE9" s="75"/>
+      <c r="BF9" s="75"/>
+      <c r="BG9" s="76" t="str">
         <f t="shared" si="3"/>
-        <v>description: "Контр_пол_ав_дебл", note: "Контроль положения переключателя аварийной деблокировки ", group: "setting", minValue: 0, maxValue: 1, step: 1, units: "null", defaultValue: 0, eventRegistration: 0</v>
+        <v>description: "Контр_пол_ав_дебл_1", note: "Контроль положения переключателя 1 аварийной деблокировки", group: "setting", minValue: 0, maxValue: 1, step: 1, units: "null", defaultValue: 0, eventRegistration: 0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16379" s="38" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="69"/>
+      <c r="B10" s="69" t="s">
+        <v>151</v>
+      </c>
+      <c r="C10" s="70"/>
+      <c r="D10" s="20" t="s">
+        <v>144</v>
+      </c>
+      <c r="E10" s="77" t="s">
+        <v>227</v>
+      </c>
+      <c r="F10" s="77" t="s">
+        <v>228</v>
+      </c>
+      <c r="G10" s="77" t="s">
+        <v>229</v>
+      </c>
+      <c r="H10" s="71" t="s">
+        <v>153</v>
+      </c>
+      <c r="I10" s="71">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="J10" s="71" t="str">
+        <f t="shared" si="1"/>
+        <v>Контр_пол_ав_дебл_2</v>
+      </c>
+      <c r="K10" s="69" t="s">
+        <v>230</v>
+      </c>
+      <c r="L10" s="72" t="s">
+        <v>62</v>
+      </c>
+      <c r="M10" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="N10" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="O10" s="70"/>
+      <c r="P10" s="73">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="73"/>
+      <c r="R10" s="70" t="s">
+        <v>65</v>
+      </c>
+      <c r="S10" s="70">
+        <v>0</v>
+      </c>
+      <c r="T10" s="70">
+        <v>1</v>
+      </c>
+      <c r="U10" s="70">
+        <v>1</v>
+      </c>
+      <c r="V10" s="70"/>
+      <c r="W10" s="70"/>
+      <c r="X10" s="70">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="70">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="74"/>
+      <c r="AA10" s="75">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="75"/>
+      <c r="AC10" s="75"/>
+      <c r="AD10" s="75"/>
+      <c r="AE10" s="75"/>
+      <c r="AF10" s="75">
+        <v>0</v>
+      </c>
+      <c r="AG10" s="75">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="75">
+        <v>0</v>
+      </c>
+      <c r="AI10" s="75"/>
+      <c r="AJ10" s="75"/>
+      <c r="AK10" s="75"/>
+      <c r="AL10" s="75"/>
+      <c r="AM10" s="75"/>
+      <c r="AN10" s="75"/>
+      <c r="AO10" s="75"/>
+      <c r="AP10" s="75"/>
+      <c r="AQ10" s="75"/>
+      <c r="AR10" s="75">
+        <v>0</v>
+      </c>
+      <c r="AS10" s="75">
+        <v>0</v>
+      </c>
+      <c r="AT10" s="75">
+        <v>0</v>
+      </c>
+      <c r="AU10" s="75">
+        <v>0</v>
+      </c>
+      <c r="AV10" s="75">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AW10" s="75" t="s">
+        <v>154</v>
+      </c>
+      <c r="AX10" s="75"/>
+      <c r="AY10" s="73"/>
+      <c r="AZ10" s="75"/>
+      <c r="BA10" s="75"/>
+      <c r="BB10" s="75"/>
+      <c r="BC10" s="75"/>
+      <c r="BD10" s="75"/>
+      <c r="BE10" s="75"/>
+      <c r="BF10" s="75"/>
+      <c r="BG10" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v>description: "Контр_пол_ав_дебл_2", note: "Контроль положения переключателя 2 аварийной деблокировки", group: "setting", minValue: 0, maxValue: 1, step: 1, units: "null", defaultValue: 0, eventRegistration: 0</v>
       </c>
     </row>
   </sheetData>
@@ -60738,15 +60907,15 @@
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="39" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B3" s="40" t="s">
         <v>144</v>
@@ -60754,7 +60923,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B4" s="41">
         <v>580</v>
@@ -60762,7 +60931,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B5" s="42" t="s">
         <v>64</v>
@@ -60770,15 +60939,15 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="43" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="43" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B7" s="42">
         <v>1</v>
@@ -60786,15 +60955,15 @@
     </row>
     <row r="8" spans="1:2" s="46" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="45" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="1:2" s="46" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="45" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B9" s="45"/>
     </row>
@@ -60803,12 +60972,12 @@
         <v>144</v>
       </c>
       <c r="B10" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="46" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="45" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B11" s="45"/>
     </row>

</xml_diff>